<commit_message>
Add multiple data management plans for various research projects
- Introduced sample data management plans covering data sharing, preservation, and access protocols.
- Included detailed descriptions of data types, roles and responsibilities, and policies for access and sharing.
- Ensured compliance with institutional guidelines and best practices for data management across different research contexts.
- Highlighted the importance of metadata standards, data formats, and archiving strategies for long-term data accessibility.
</commit_message>
<xml_diff>
--- a/data/input/Rules.xlsx
+++ b/data/input/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nahid\dmpbridge\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{946844D6-A169-4B0C-AAD4-CAB677C0F4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0440C19A-41F8-40BA-8BB4-7E1B935520FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="15">
   <si>
     <t>#</t>
   </si>
@@ -54,15 +54,9 @@
     <t>N</t>
   </si>
   <si>
-    <t>Copy "section.description" into "question.text" AND "section.title"</t>
-  </si>
-  <si>
     <t>Copy "section.title" into "question.text"</t>
   </si>
   <si>
-    <t>Copy "question.text" into "section.title"</t>
-  </si>
-  <si>
     <t>Legend:</t>
   </si>
   <si>
@@ -73,6 +67,9 @@
   </si>
   <si>
     <t>Copy title into "question.text"</t>
+  </si>
+  <si>
+    <t>Copy "section.description" into "question.text"</t>
   </si>
 </sst>
 </file>
@@ -453,7 +450,7 @@
         <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -473,7 +470,7 @@
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -493,7 +490,7 @@
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -513,7 +510,7 @@
         <v>6</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -533,7 +530,7 @@
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -553,7 +550,7 @@
         <v>6</v>
       </c>
       <c r="F8" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -593,7 +590,7 @@
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -613,7 +610,7 @@
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -633,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="F12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -653,7 +650,7 @@
         <v>8</v>
       </c>
       <c r="F13" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -673,7 +670,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -693,7 +690,7 @@
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -713,7 +710,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -738,13 +735,13 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -752,7 +749,7 @@
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor data management plan samples and update annotation rules
- Deleted multiple sample JSON files (sample6.json, sample7.json, sample8.json, sample9.json) from the data management plan output directory.
- Updated the annotation rules in `annotation_rules.py` to improve clarity and maintainability, including changes to the handling of empty fields and the order of precedence for filling question text.
- Modified test cases in `test_annotation_rules.py` to reflect the new logic in the annotation rules, ensuring that the tests accurately validate the expected behavior of the system.
- Enhanced documentation within the code to clarify the purpose and functionality of the annotation rules and their application.
</commit_message>
<xml_diff>
--- a/data/input/Rules.xlsx
+++ b/data/input/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nahid\dmpbridge\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0440C19A-41F8-40BA-8BB4-7E1B935520FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBB67D8-1BD5-46FD-A5DC-D89E95756A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -390,6 +390,8 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="4" width="25.5703125" customWidth="1"/>
+    <col min="5" max="5" width="35.140625" customWidth="1"/>
     <col min="6" max="6" width="89.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -401,13 +403,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Update build report and add new sample data for llama3.3-70b model
- Revised the build report to reflect the completion of all experiments and updated results for the models.
- Enhanced the analysis of model performance, highlighting the changes in scoring and runtime.
- Added new labeled and structured JSON output files for sample 10 of the llama3.3-70b model, detailing data management practices and accessibility.
- Included comprehensive sections on policy, scope, data format, accessibility, derivative products, and archiving in the new output files.
</commit_message>
<xml_diff>
--- a/data/input/Rules.xlsx
+++ b/data/input/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nahid\dmpbridge\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBB67D8-1BD5-46FD-A5DC-D89E95756A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{633A3500-934C-44B0-AF4B-965D972630A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="16">
   <si>
     <t>#</t>
   </si>
@@ -66,10 +66,13 @@
     <t>= non-empty (has a value)</t>
   </si>
   <si>
-    <t>Copy title into "question.text"</t>
-  </si>
-  <si>
     <t>Copy "section.description" into "question.text"</t>
+  </si>
+  <si>
+    <t>Copy "section.description" into "question.text" and "section.title"</t>
+  </si>
+  <si>
+    <t>Copy title into "question.text" and "section.title"</t>
   </si>
 </sst>
 </file>
@@ -592,7 +595,7 @@
         <v>6</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -632,7 +635,7 @@
         <v>6</v>
       </c>
       <c r="F12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>